<commit_message>
feat: complete AdmitFlow v2 analytics platform
</commit_message>
<xml_diff>
--- a/TRACKER.xlsx
+++ b/TRACKER.xlsx
@@ -21,7 +21,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -60,11 +62,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -537,8 +540,6 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>docs/PROJECT_SPEC.md</t>
@@ -546,7 +547,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Initial project scope defined.</t>
+          <t>Scope and deliverables documented.</t>
         </is>
       </c>
     </row>
@@ -584,8 +585,6 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
           <t>docs/ARCHITECTURE.md</t>
@@ -593,7 +592,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Core architecture documented.</t>
+          <t>Architecture matches the implemented local stack.</t>
         </is>
       </c>
     </row>
@@ -631,8 +630,6 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>docs/DEVELOPMENT_PLAN.md</t>
@@ -640,7 +637,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Milestones defined.</t>
+          <t>Milestone plan retained.</t>
         </is>
       </c>
     </row>
@@ -678,8 +675,6 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
           <t>docs/ACCEPTANCE_CRITERIA.md</t>
@@ -687,7 +682,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Verification criteria established.</t>
+          <t>Acceptance gates retained and reconciled in final verification.</t>
         </is>
       </c>
     </row>
@@ -725,16 +720,14 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
-          <t>evidence/README.md</t>
+          <t>evidence/README.md; docs/EVIDENCE.md</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Evidence policy documented.</t>
+          <t>Evidence policy and artifact map documented.</t>
         </is>
       </c>
     </row>
@@ -769,15 +762,17 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>.git; Git history</t>
+        </is>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Git repository will be initialized during setup.</t>
+          <t>Repository initialized; implementation and verification milestone recorded in Git history.</t>
         </is>
       </c>
     </row>
@@ -812,15 +807,17 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>evidence/dataset/dataset_summary.json; evidence/dataset/validation_report.json</t>
+        </is>
+      </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Dataset work begins after foundation verification.</t>
+          <t>Fixed-seed 4,200-row dataset passes validation.</t>
         </is>
       </c>
     </row>
@@ -855,15 +852,17 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>evidence/metrics/analytics_report.json</t>
+        </is>
+      </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Requires generated dataset.</t>
+          <t>Cumulative funnel analytics generated from current dataset.</t>
         </is>
       </c>
     </row>
@@ -898,15 +897,17 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>evidence/metrics/analytics_report.json</t>
+        </is>
+      </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Requires validated dataset.</t>
+          <t>Cycle, programme, region, and selectivity cohorts generated.</t>
         </is>
       </c>
     </row>
@@ -941,15 +942,17 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>evidence/metrics/analytics_report.json</t>
+        </is>
+      </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Must avoid causal claims.</t>
+          <t>Campaign attribution is explicitly descriptive, not causal.</t>
         </is>
       </c>
     </row>
@@ -984,15 +987,17 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>evidence/models/model_report.json; evidence/models/admitflow_model.joblib</t>
+        </is>
+      </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Model metrics to be captured from execution.</t>
+          <t>Training and feature summaries captured. Predictive quality is weak; models are not decision-ready.</t>
         </is>
       </c>
     </row>
@@ -1027,15 +1032,17 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>evidence/metrics/forecast_report.json</t>
+        </is>
+      </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Temporal leakage checks required.</t>
+          <t>H1/H2/H4/H6 evaluated; only six annual observations are available.</t>
         </is>
       </c>
     </row>
@@ -1070,15 +1077,17 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>evidence/metrics/scenario_report.json; evidence/api/api_smoke.json</t>
+        </is>
+      </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Scenario outputs must be deterministic.</t>
+          <t>Deterministic scenario engine and authenticated route verified.</t>
         </is>
       </c>
     </row>
@@ -1113,15 +1122,17 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>evidence/api/api_smoke.json; evidence/security/auth_check.json</t>
+        </is>
+      </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Includes auth and audit flows.</t>
+          <t>Protected API routes and missing-token rejection verified; audit log is process-local.</t>
         </is>
       </c>
     </row>
@@ -1156,15 +1167,17 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>evidence/screenshots/dashboard.png; evidence/screenshots/dashboard-mobile.png; evidence/screenshots/scenario.png; evidence/tests/frontend_vitest.txt</t>
+        </is>
+      </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Must include light/dark theme.</t>
+          <t>Desktop/mobile dashboard and live scenario captured; interactions covered by Vitest.</t>
         </is>
       </c>
     </row>
@@ -1199,15 +1212,17 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>evidence/tests/backend_pytest.txt; evidence/tests/frontend_vitest.txt; evidence/tests/frontend_lint.txt; evidence/tests/frontend_build.txt</t>
+        </is>
+      </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Evidence required before final verification.</t>
+          <t>Automated suites pass; production build has a disclosed chunk-size warning.</t>
         </is>
       </c>
     </row>
@@ -1242,15 +1257,17 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>docs/FINAL_PROJECT_REPORT.md; docs/FINAL_VERIFICATION.md</t>
+        </is>
+      </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Final evidence must be linked.</t>
+          <t>Final documentation completed with evidence and limitations.</t>
         </is>
       </c>
     </row>
@@ -1265,7 +1282,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1314,6 +1331,36 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>CLOSEOUT</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Project Agent</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Final local verification and evidence capture</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>docs/FINAL_VERIFICATION.md</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Automated checks pass; model limitations recorded.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1325,7 +1372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1386,6 +1433,681 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AF-E01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>A7</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Execution artifact</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Dataset validation</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>evidence/dataset/validation_report.json</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Automated local run</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>4,200 rows; no validation issues.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AF-E02</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>A8</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Execution artifact</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Analytics report</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>evidence/metrics/analytics_report.json</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Automated local run</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Dashboard, funnel, cohorts, programme, and attribution outputs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>AF-E03</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>A11</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Execution artifact</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Model report and artifact</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>evidence/models/model_report.json; evidence/models/admitflow_model.joblib</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>GENERATED_WITH_LIMITATIONS</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Automated local run</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Random forest predicts no positives at threshold 0.5; not decision-ready.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AF-E04</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>A12</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Execution artifact</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Forecast report</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>evidence/metrics/forecast_report.json</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>PASS_WITH_LIMITATIONS</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Automated local run</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Two-year holdout over six annual observations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AF-E05</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>A13</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Execution artifact</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Scenario report</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>evidence/metrics/scenario_report.json</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Automated local run</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Deterministic baseline/scenario/delta output.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>AF-E06</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>A14</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Execution artifact</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>API smoke report</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>evidence/api/api_smoke.json</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Automated local run</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>10/10 authenticated API operations successful.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>AF-E07</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>A14</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Execution artifact</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Auth boundary report</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>evidence/security/auth_check.json</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Automated local run</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>401 without token; token/password omitted from report.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>AF-E08</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>A15</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Execution artifact</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Desktop dashboard screenshot</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>evidence/screenshots/dashboard.png</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>CAPTURED</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Automated local run</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Authenticated live dashboard at desktop viewport.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>AF-E09</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>A15</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Execution artifact</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Mobile dashboard screenshot</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>evidence/screenshots/dashboard-mobile.png</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>CAPTURED</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Automated local run</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Authenticated live dashboard at 390px viewport.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>AF-E10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>A16</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Execution artifact</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Backend test suite</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>evidence/tests/backend_pytest.txt</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Automated local run</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Current full pytest output.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>AF-E11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>A16</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Execution artifact</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Frontend test suite</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>evidence/tests/frontend_vitest.txt</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Automated local run</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Current full Vitest output.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>AF-E12</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>A16</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Execution artifact</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Frontend lint</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>evidence/tests/frontend_lint.txt</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Automated local run</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>No lint diagnostics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>AF-E13</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>A16</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Execution artifact</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Production build</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>evidence/tests/frontend_build.txt</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>PASS_WITH_WARNING</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Automated local run</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Build succeeds; bundle exceeds 500 kB warning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>AF-E14</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>A17</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Execution artifact</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Final verification documents</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>docs/FINAL_VERIFICATION.md; docs/FINAL_PROJECT_REPORT.md</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Automated local run</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Status and limitations stated explicitly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>AF-E15</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>A15</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Execution artifact</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Scaled scenario screenshot</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>evidence/screenshots/scenario.png</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>CAPTURED</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Automated local run</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Live UI scenario at twice the baseline application volume; stage totals and changes shown.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1397,7 +2119,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1452,6 +2174,216 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AF-T01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>A16</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Backend pytest suite</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>python -m pytest -q</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>All tests pass</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>16 passed; 0 failed</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>evidence/tests/backend_pytest.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AF-T02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>A16</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Frontend Vitest suite</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>npm test</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>All tests pass</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>3 passed</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>evidence/tests/frontend_vitest.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>AF-T03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>A16</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Frontend lint</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>npm run lint</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>No diagnostics</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Clean</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>evidence/tests/frontend_lint.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AF-T04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>A16</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Frontend production build</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>npm run build</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Build succeeds</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Build succeeded; bundle-size warning present</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>PASS_WITH_WARNING</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>evidence/tests/frontend_build.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AF-T05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>A14</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Authenticated API smoke checks</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>python scripts/capture_evidence.py</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Protected routes respond successfully</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>10/10 operations successful</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>evidence/api/api_smoke.json</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1463,7 +2395,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1509,6 +2441,76 @@
       <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Logistic Regression</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>data/admission_data.csv (synthetic)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>enrolled</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>{"roc_auc": 0.5573, "pr_auc": 0.0964, "accuracy": 0.6143, "precision": 0.1028, "recall": 0.4659, "f1": 0.1684}</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>evidence/models/model_report.json; evidence/models/admitflow_model.joblib</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Evaluated; not decision-ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Random Forest</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>data/admission_data.csv (synthetic)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>enrolled</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>{"roc_auc": 0.5195, "pr_auc": 0.1037, "accuracy": 0.9162, "precision": 0.0, "recall": 0.0, "f1": 0.0}</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>evidence/models/model_report.json; evidence/models/admitflow_model.joblib</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Evaluated; not decision-ready</t>
         </is>
       </c>
     </row>
@@ -1559,7 +2561,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>5</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4">
@@ -1569,7 +2571,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -1589,7 +2591,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -1599,7 +2601,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="8">
@@ -1608,7 +2610,6 @@
           <t>total recorded actual hours</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1617,7 +2618,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10">
@@ -1627,7 +2628,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11">

</xml_diff>